<commit_message>
archive: preserve finite-frame HLS experiment and streaming contract
</commit_message>
<xml_diff>
--- a/Viet/docs/hardware_architecture.xlsx
+++ b/Viet/docs/hardware_architecture.xlsx
@@ -73,6 +73,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -94,18 +95,21 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFC9211E"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="9">
@@ -199,56 +203,60 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -443,404 +451,404 @@
         <v>0</v>
       </c>
       <c r="M3" s="1"/>
-      <c r="N3" s="0" t="s">
+      <c r="N3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="D4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="J4" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M4" s="2" t="n">
+      <c r="M4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="2" t="n">
+      <c r="O4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="P4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q4" s="2" t="n">
+      <c r="P4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="R4" s="2" t="n">
+      <c r="R4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="S4" s="2" t="n">
+      <c r="S4" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="T4" s="2" t="n">
+      <c r="T4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="U4" s="2" t="n">
+      <c r="U4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="V4" s="2" t="n">
+      <c r="V4" s="3" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="J5" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M5" s="2" t="n">
+      <c r="L5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M5" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="N5" s="2" t="n">
+      <c r="N5" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="O5" s="2" t="n">
+      <c r="O5" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="P5" s="2" t="n">
+      <c r="P5" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="Q5" s="2" t="n">
+      <c r="Q5" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="R5" s="2" t="n">
+      <c r="R5" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="S5" s="2" t="n">
+      <c r="S5" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="T5" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="U5" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="V5" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="J6" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="M6" s="2" t="n">
+      <c r="M6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N6" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O6" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="P6" s="2" t="n">
+      <c r="P6" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="Q6" s="2" t="n">
+      <c r="Q6" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="R6" s="2" t="n">
+      <c r="R6" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="S6" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="T6" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="U6" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="V6" s="3" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="N7" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="O7" s="2" t="n">
+      <c r="O7" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="P7" s="2" t="n">
+      <c r="P7" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="Q7" s="2" t="n">
+      <c r="Q7" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="R7" s="2" t="n">
+      <c r="R7" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="S7" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="T7" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="U7" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="V7" s="3" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>44</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="J8" s="3" t="n">
         <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>54</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>55</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="3" t="n">
         <v>57</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="J9" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M10" s="2" t="n">
+      <c r="M10" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="N10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="O10" s="2" t="n">
+      <c r="O10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="P10" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q10" s="2" t="n">
+      <c r="P10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="R10" s="2" t="n">
+      <c r="R10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="S10" s="2" t="n">
+      <c r="S10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="T10" s="2" t="n">
+      <c r="T10" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="U10" s="2" t="n">
+      <c r="U10" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="V10" s="2" t="n">
+      <c r="V10" s="3" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M11" s="2" t="n">
+      <c r="L11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M11" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="N11" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="O11" s="2" t="n">
+      <c r="O11" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="P11" s="2" t="n">
+      <c r="P11" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="Q11" s="2" t="n">
+      <c r="Q11" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="R11" s="2" t="n">
+      <c r="R11" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="S11" s="2" t="n">
+      <c r="S11" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="T11" s="2" t="n">
+      <c r="T11" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="U11" s="2" t="n">
+      <c r="U11" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V11" s="2" t="n">
+      <c r="V11" s="3" t="n">
         <v>19</v>
       </c>
     </row>
@@ -849,851 +857,851 @@
         <v>7</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="2" t="s">
         <v>1</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="I12" s="1"/>
-      <c r="L12" s="3" t="s">
+      <c r="L12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="M12" s="2" t="n">
+      <c r="M12" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="N12" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="O12" s="2" t="n">
+      <c r="O12" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="P12" s="2" t="n">
+      <c r="P12" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="Q12" s="2" t="n">
+      <c r="Q12" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="R12" s="2" t="n">
+      <c r="R12" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="S12" s="2" t="n">
+      <c r="S12" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="T12" s="2" t="n">
+      <c r="T12" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="U12" s="2" t="n">
+      <c r="U12" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="V12" s="2" t="n">
+      <c r="V12" s="3" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="4" t="n">
+      <c r="D13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="J13" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="L13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M13" s="2" t="n">
+      <c r="M13" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N13" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="O13" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="P13" s="2" t="n">
+      <c r="P13" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="Q13" s="2" t="n">
+      <c r="Q13" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="R13" s="2" t="n">
+      <c r="R13" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="S13" s="2" t="n">
+      <c r="S13" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="T13" s="2" t="n">
+      <c r="T13" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="U13" s="2" t="n">
+      <c r="U13" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V13" s="2" t="n">
+      <c r="V13" s="3" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="F14" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="H14" s="8" t="n">
+      <c r="F14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="I14" s="9" t="n">
+      <c r="I14" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="9" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I15" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="N15" s="0" t="s">
+      <c r="N15" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L16" s="3" t="s">
+      <c r="L16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M16" s="2" t="n">
+      <c r="M16" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="N16" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="O16" s="2" t="n">
+      <c r="O16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="P16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q16" s="2" t="n">
+      <c r="P16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="R16" s="2" t="n">
+      <c r="R16" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="S16" s="2" t="n">
+      <c r="S16" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="T16" s="2" t="n">
+      <c r="T16" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="U16" s="2" t="n">
+      <c r="U16" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="V16" s="2" t="n">
+      <c r="V16" s="3" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L17" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="2" t="n">
+      <c r="L17" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="N17" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="O17" s="2" t="n">
+      <c r="O17" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="P17" s="2" t="n">
+      <c r="P17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="Q17" s="2" t="n">
+      <c r="Q17" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="R17" s="2" t="n">
+      <c r="R17" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="S17" s="2" t="n">
+      <c r="S17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="T17" s="2" t="n">
+      <c r="T17" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="U17" s="2" t="n">
+      <c r="U17" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V17" s="2" t="n">
+      <c r="V17" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D18" s="4" t="n">
+      <c r="C18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="F18" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="J18" s="7" t="n">
+      <c r="I18" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="L18" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M18" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="N18" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="O18" s="2" t="n">
+      <c r="O18" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="P18" s="2" t="n">
+      <c r="P18" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="Q18" s="2" t="n">
+      <c r="Q18" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="R18" s="2" t="n">
+      <c r="R18" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="S18" s="2" t="n">
+      <c r="S18" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="T18" s="2" t="n">
+      <c r="T18" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="U18" s="2" t="n">
+      <c r="U18" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="V18" s="2" t="n">
+      <c r="V18" s="3" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="F19" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="H19" s="8" t="n">
+      <c r="F19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H19" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="I19" s="9" t="n">
+      <c r="I19" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="L19" s="3" t="s">
+      <c r="L19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M19" s="2" t="n">
+      <c r="M19" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="N19" s="2" t="n">
+      <c r="N19" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="O19" s="2" t="n">
+      <c r="O19" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="P19" s="2" t="n">
+      <c r="P19" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="Q19" s="2" t="n">
+      <c r="Q19" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="R19" s="2" t="n">
+      <c r="R19" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="S19" s="2" t="n">
+      <c r="S19" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="T19" s="2" t="n">
+      <c r="T19" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="U19" s="2" t="n">
+      <c r="U19" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V19" s="2" t="n">
+      <c r="V19" s="3" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="D20" s="12" t="n">
+      <c r="D20" s="13" t="n">
         <v>44</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="F20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H20" s="7" t="n">
+      <c r="H20" s="8" t="n">
         <v>41</v>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I20" s="7" t="n">
         <v>43</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="6" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N21" s="0" t="s">
+      <c r="N21" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M22" s="2" t="n">
+      <c r="M22" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="N22" s="2" t="n">
+      <c r="N22" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="O22" s="2" t="n">
+      <c r="O22" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="P22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q22" s="2" t="n">
+      <c r="P22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q22" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="R22" s="2" t="n">
+      <c r="R22" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="S22" s="2" t="n">
+      <c r="S22" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="T22" s="2" t="n">
+      <c r="T22" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="U22" s="2" t="n">
+      <c r="U22" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="V22" s="2" t="n">
+      <c r="V22" s="3" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B23" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C23" s="4" t="n">
+      <c r="B23" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="F23" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H23" s="5" t="n">
+      <c r="H23" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="I23" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="J23" s="7" t="n">
+      <c r="J23" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="L23" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="2" t="n">
+      <c r="L23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N23" s="2" t="n">
+      <c r="N23" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="O23" s="2" t="n">
+      <c r="O23" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="P23" s="2" t="n">
+      <c r="P23" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="Q23" s="2" t="n">
+      <c r="Q23" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="R23" s="2" t="n">
+      <c r="R23" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="S23" s="2" t="n">
+      <c r="S23" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="T23" s="2" t="n">
+      <c r="T23" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="U23" s="2" t="n">
+      <c r="U23" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V23" s="2" t="n">
+      <c r="V23" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="F24" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="H24" s="8" t="n">
+      <c r="F24" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="I24" s="9" t="n">
+      <c r="I24" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J24" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="L24" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="M24" s="2" t="n">
+      <c r="M24" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="N24" s="2" t="n">
+      <c r="N24" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="O24" s="2" t="n">
+      <c r="O24" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="P24" s="2" t="n">
+      <c r="P24" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="Q24" s="2" t="n">
+      <c r="Q24" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="R24" s="2" t="n">
+      <c r="R24" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="S24" s="2" t="n">
+      <c r="S24" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="T24" s="2" t="n">
+      <c r="T24" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="U24" s="2" t="n">
+      <c r="U24" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="V24" s="2" t="n">
+      <c r="V24" s="3" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="11" t="n">
         <v>42</v>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C25" s="13" t="n">
         <v>44</v>
       </c>
-      <c r="D25" s="12" t="n">
+      <c r="D25" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="E25" s="11" t="n">
+      <c r="E25" s="12" t="n">
         <v>46</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="F25" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H25" s="7" t="n">
+      <c r="H25" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="I25" s="6" t="n">
+      <c r="I25" s="7" t="n">
         <v>44</v>
       </c>
-      <c r="J25" s="5" t="n">
+      <c r="J25" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="L25" s="3" t="s">
+      <c r="L25" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M25" s="2" t="n">
+      <c r="M25" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="N25" s="2" t="n">
+      <c r="N25" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="O25" s="2" t="n">
+      <c r="O25" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="P25" s="2" t="n">
+      <c r="P25" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="Q25" s="2" t="n">
+      <c r="Q25" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="R25" s="2" t="n">
+      <c r="R25" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="S25" s="2" t="n">
+      <c r="S25" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="T25" s="2" t="n">
+      <c r="T25" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="U25" s="2" t="n">
+      <c r="U25" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V25" s="2" t="n">
+      <c r="V25" s="3" t="n">
         <v>39</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N27" s="0" t="s">
+      <c r="N27" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B28" s="4" t="n">
+      <c r="A28" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="D28" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="F28" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H28" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I28" s="6" t="n">
+      <c r="H28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="J28" s="7" t="n">
+      <c r="J28" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="L28" s="3" t="s">
+      <c r="L28" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M28" s="2" t="n">
+      <c r="M28" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="N28" s="2" t="n">
+      <c r="N28" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="2" t="n">
+      <c r="O28" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="P28" s="2" t="n">
+      <c r="P28" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="Q28" s="2" t="n">
+      <c r="Q28" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="R28" s="2" t="n">
+      <c r="R28" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="S28" s="2" t="n">
+      <c r="S28" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="T28" s="2" t="n">
+      <c r="T28" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="U28" s="2" t="n">
+      <c r="U28" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="V28" s="2" t="n">
+      <c r="V28" s="3" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="F29" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="H29" s="8" t="n">
+      <c r="F29" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H29" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="I29" s="9" t="n">
+      <c r="I29" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="J29" s="8" t="n">
+      <c r="J29" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="L29" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="M29" s="2" t="n">
+      <c r="L29" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M29" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="N29" s="2" t="n">
+      <c r="N29" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="O29" s="2" t="n">
+      <c r="O29" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="P29" s="2" t="n">
+      <c r="P29" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="Q29" s="2" t="n">
+      <c r="Q29" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="R29" s="2" t="n">
+      <c r="R29" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="S29" s="2" t="n">
+      <c r="S29" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="T29" s="2" t="n">
+      <c r="T29" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="U29" s="2" t="n">
+      <c r="U29" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V29" s="2" t="n">
+      <c r="V29" s="3" t="n">
         <v>19</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="11" t="n">
         <v>43</v>
       </c>
-      <c r="B30" s="12" t="n">
+      <c r="B30" s="13" t="n">
         <v>44</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="13" t="n">
         <v>45</v>
       </c>
-      <c r="D30" s="12" t="n">
+      <c r="D30" s="13" t="n">
         <v>46</v>
       </c>
-      <c r="E30" s="11" t="n">
+      <c r="E30" s="12" t="n">
         <v>47</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="F30" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H30" s="7" t="n">
+      <c r="H30" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="I30" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="L30" s="3" t="s">
+      <c r="L30" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="M30" s="2" t="n">
+      <c r="M30" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="N30" s="2" t="n">
+      <c r="N30" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="O30" s="2" t="n">
+      <c r="O30" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="P30" s="2" t="n">
+      <c r="P30" s="3" t="n">
         <v>33</v>
       </c>
-      <c r="Q30" s="2" t="n">
+      <c r="Q30" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="R30" s="2" t="n">
+      <c r="R30" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="S30" s="2" t="n">
+      <c r="S30" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="T30" s="2" t="n">
+      <c r="T30" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="U30" s="2" t="n">
+      <c r="U30" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="V30" s="2" t="n">
+      <c r="V30" s="3" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L31" s="3" t="s">
+      <c r="L31" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M31" s="2" t="n">
+      <c r="M31" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="N31" s="2" t="n">
+      <c r="N31" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="O31" s="2" t="n">
+      <c r="O31" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="P31" s="2" t="n">
+      <c r="P31" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="Q31" s="2" t="n">
+      <c r="Q31" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="R31" s="2" t="n">
+      <c r="R31" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="S31" s="2" t="n">
+      <c r="S31" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="T31" s="2" t="n">
+      <c r="T31" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="U31" s="2" t="n">
+      <c r="U31" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="V31" s="2" t="n">
+      <c r="V31" s="3" t="n">
         <v>39</v>
       </c>
     </row>

</xml_diff>